<commit_message>
Wed Apr  1 10:35:16 PM CEST 2026
</commit_message>
<xml_diff>
--- a/exams-summer2026.xlsx
+++ b/exams-summer2026.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">Date esami estate 2026</t>
   </si>
@@ -63,6 +63,9 @@
     <t xml:space="preserve">10/07/2026 15:00</t>
   </si>
   <si>
+    <t>&lt;&lt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">07/09/2026 15:00</t>
   </si>
   <si>
@@ -93,22 +96,22 @@
     <t xml:space="preserve">28/08/2026 15:00</t>
   </si>
   <si>
+    <t xml:space="preserve">QUANTUM PHYSICS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17/06/2026 11:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/07/2026 11:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/09/2026 11:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">APPLIED STATISTICS</t>
   </si>
   <si>
     <t>tba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUANTUM PHYSICS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17/06/2026 11:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/07/2026 11:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09/09/2026 11:30</t>
   </si>
   <si>
     <t xml:space="preserve"> NUMERICAL METHODS FOR PARTIAL DIFFERENTIAL EQUATIONS</t>
@@ -166,7 +169,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -262,11 +265,20 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thick">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -302,26 +314,20 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="3" borderId="6" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf fontId="3" fillId="3" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="6" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="6" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="5" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="7" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="3" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf fontId="3" fillId="0" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -909,116 +915,122 @@
       <c r="B10" s="10" t="s">
         <v>14</v>
       </c>
+      <c r="C10" s="19" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" s="11"/>
       <c r="B11" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="19" t="s">
         <v>17</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" s="15"/>
-      <c r="B13" s="20" t="s">
-        <v>18</v>
+      <c r="B13" s="16" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" s="17"/>
       <c r="B14" s="21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="9"/>
-      <c r="B16" s="24" t="s">
-        <v>23</v>
+      <c r="B16" s="10" t="s">
+        <v>24</v>
       </c>
       <c r="C16" s="23"/>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" s="11"/>
-      <c r="B17" s="25" t="s">
-        <v>24</v>
+      <c r="B17" s="12" t="s">
+        <v>25</v>
       </c>
       <c r="C17" s="23"/>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="26" t="s">
+      <c r="A18" s="24" t="s">
         <v>26</v>
       </c>
+      <c r="B18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="25"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16" t="s">
-        <v>26</v>
-      </c>
+      <c r="A19" s="24"/>
+      <c r="B19" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="25"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18" t="s">
-        <v>26</v>
-      </c>
+      <c r="A20" s="24"/>
+      <c r="B20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="25"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>28</v>
+      <c r="A21" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="27" t="s">
-        <v>29</v>
+      <c r="A22" s="15"/>
+      <c r="B22" s="16" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="11"/>
-      <c r="B23" s="25" t="s">
-        <v>30</v>
+      <c r="A23" s="17"/>
+      <c r="B23" s="18" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="26" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="29"/>
+      <c r="A25" s="15"/>
       <c r="B25" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="30"/>
+      <c r="A26" s="17"/>
       <c r="B26" s="18" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>